<commit_message>
Automatická aktualizace překladové databáze z webové aplikace
</commit_message>
<xml_diff>
--- a/translate-PL.xlsx
+++ b/translate-PL.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B316"/>
+  <dimension ref="A1:B317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4209,6 +4209,18 @@
       <c r="B316" t="inlineStr">
         <is>
           <t>LPO 25 + SZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Dětská postel DOPLO PINE s přistýlkou, zábranou, rošty  + ŠUPLÍKY</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>LPW 01 + SZ</t>
         </is>
       </c>
     </row>

</xml_diff>